<commit_message>
Enhance project configuration and documentation
- Updated .gitignore to exclude data and debug logs directories.
- Added batch_size and max_retries parameters to config.yaml for improved order processing.
- Enhanced document.html with new sections for CDP mode and debugging, and updated usage descriptions.
- Refined main.py to incorporate batch processing and auto-retry logic for order handling.
- Updated sample_orders.xlsx to reflect new order structure.
- Introduced new UI/UX design intelligence skill with comprehensive guidelines and resources.
</commit_message>
<xml_diff>
--- a/sample_orders.xlsx
+++ b/sample_orders.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/lap13978-local/work/code/src/github/bot-mua-hang/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{7A55B35C-3F81-DE4F-8B48-3C29369DFC20}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{AEC58D9D-82A4-534D-A195-392BA31B4E50}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="0" yWindow="760" windowWidth="30240" windowHeight="18880" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -20,7 +20,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="13" uniqueCount="13">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="29" uniqueCount="26">
   <si>
     <t>product_url</t>
   </si>
@@ -32,6 +32,12 @@
   </si>
   <si>
     <t>quantity</t>
+  </si>
+  <si>
+    <t>https://shopee.vn/%E1%BB%90p-L%C6%B0ng-Iphone-Silicon-D%E1%BA%BBo-Camera-Nh%C3%A1m-M%E1%BB%9D-N%C3%A2ng-C%E1%BA%A5p-L%C3%AAn-IP-17-11-12-13-14-15-16-17-pro-max-plus-promax-Awifi-X5-1-i.7669738.57555754369</t>
+  </si>
+  <si>
+    <t>Ốp Lưng Iphone Silicon Dẻo Camera Nhám Mờ Nâng Cấp Lên IP 17 11/12/13/14/15/16/17/pro/max/plus/promax - Awifi X5-1</t>
   </si>
   <si>
     <t>receiver_phone_number</t>
@@ -60,6 +66,39 @@
   </si>
   <si>
     <t>Màu đen, size M</t>
+  </si>
+  <si>
+    <t>Nhóm màu: Trắng Mờ Camera Lớn, Dòng máy: IP11</t>
+  </si>
+  <si>
+    <t>https://shopee.vn/Tawii.-T%C3%BAi-%C4%91eo-ch%C3%A9o-nam-T%C3%BAi-nam-UNISEX-T%C3%BAi-%C4%91a-n%C4%83ng-nhi%E1%BB%81u-C%C3%B4ng-su%E1%BA%A5t-l%E1%BB%9Bn-C%C3%B3-th%E1%BB%83-c%C3%A0i-%C4%91%E1%BA%B7t-m%C3%A1y-t%C3%ADnh-i.1613670694.56052771445?extraParams=%7B%22display_model_id%22%3A254112951495%2C%22model_selection_logic%22%3A3%7D&amp;sp_atk=9be0be2a-d5c0-472b-a523-2a3556f764a0&amp;xptdk=9be0be2a-d5c0-472b-a523-2a3556f764a0</t>
+  </si>
+  <si>
+    <t>Màu sắc: Be</t>
+  </si>
+  <si>
+    <t>Tawii. Túi đeo chéo nam Túi nam UNISEX Túi đa năng nhiều Công suất lớn Có thể cài đặt máy tính</t>
+  </si>
+  <si>
+    <t>https://shopee.vn/-AMINO-MICELLAR-M%E1%BB%9AI-N%C6%B0%E1%BB%9Bc-t%E1%BA%A9y-trang-l%C3%A0m-s%E1%BA%A1ch-s%C3%A2u-lo%E1%BA%A1i-b%E1%BB%8F-b%E1%BB%A5i-b%E1%BA%A9n-trang-%C4%91i%E1%BB%83m-3-in-1-L'Oreal-Paris-Micellar-Water-400ml-i.37251933.591989399?extraParams=%7B%22display_model_id%22%3A1161019774%2C%22model_selection_logic%22%3A3%7D</t>
+  </si>
+  <si>
+    <t>[AMINO MICELLAR MỚI] Nước tẩy trang làm sạch sâu, loại bỏ bụi bẩn &amp; trang điểm 3-in-1 L'Oreal Paris Micellar Water 400ml</t>
+  </si>
+  <si>
+    <t>Color: Amino Acid</t>
+  </si>
+  <si>
+    <t>https://shopee.vn/S%E1%BB%AFa-d%C6%B0%E1%BB%A1ng-%E1%BA%A9m-ph%E1%BB%A5c-h%E1%BB%93i-chuy%C3%AAn-s%C3%A2u-v%C3%A0-gi%E1%BB%AF-da-%E1%BA%A9m-m%E1%BB%8Bn-su%E1%BB%91t-48H-duy-tr%C3%AC-h%C3%A0ng-r%C3%A0o-b%E1%BA%A3o-v%E1%BB%87-da-CERAVE-MOISTURISING-LOTION-236ML-i.812449960.21033321173?extraParams=%7B%22display_model_id%22%3A68998706452%2C%22model_selection_logic%22%3A3%7D</t>
+  </si>
+  <si>
+    <t>Sữa dưỡng ẩm phục hồi chuyên sâu và giữ da ẩm mịn suốt 48H, duy trì hàng rào bảo vệ da CERAVE MOISTURISING LOTION</t>
+  </si>
+  <si>
+    <t>https://shopee.vn/-MUA-2-GI%E1%BA%A2M-45-Combo-2-t%C3%BAi-Refill-C%C3%A0-ph%C3%AA-%C4%90%E1%BA%AFk-L%E1%BA%AFk-l%C3%A0m-s%E1%BA%A1ch-da-ch%E1%BA%BFt-c%C6%A1-th%E1%BB%83-Cocoon-600ml-i.175753395.25114824196?extraParams=%7B%22display_model_id%22%3A255364173361%2C%22model_selection_logic%22%3A3%7D</t>
+  </si>
+  <si>
+    <t>[MUA 2 GIẢM 45%] Combo 2 túi Refill - Cà phê Đắk Lắk làm sạch da chết cơ thể Cocoon 600ml</t>
   </si>
 </sst>
 </file>
@@ -413,7 +452,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:H2"/>
+  <dimension ref="A1:H7"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="15" x14ac:dyDescent="0.2"/>
   <cols>
     <col min="1" max="1" width="54.1640625" customWidth="1"/>
@@ -432,50 +471,127 @@
         <v>1</v>
       </c>
       <c r="C1" t="s">
-        <v>11</v>
+        <v>13</v>
       </c>
       <c r="D1" t="s">
         <v>2</v>
       </c>
       <c r="E1" t="s">
-        <v>4</v>
+        <v>6</v>
       </c>
       <c r="F1" t="s">
-        <v>5</v>
+        <v>7</v>
       </c>
       <c r="G1" t="s">
         <v>3</v>
       </c>
       <c r="H1" t="s">
-        <v>7</v>
+        <v>9</v>
       </c>
     </row>
     <row r="2" spans="1:8" ht="32" x14ac:dyDescent="0.2">
       <c r="A2" s="1" t="s">
-        <v>9</v>
+        <v>11</v>
       </c>
       <c r="B2" s="2" t="s">
+        <v>12</v>
+      </c>
+      <c r="C2" t="s">
+        <v>14</v>
+      </c>
+      <c r="D2" t="s">
         <v>10</v>
-      </c>
-      <c r="C2" t="s">
-        <v>12</v>
-      </c>
-      <c r="D2" t="s">
-        <v>8</v>
       </c>
       <c r="E2">
         <v>976633782</v>
       </c>
       <c r="F2" t="s">
-        <v>6</v>
+        <v>8</v>
       </c>
       <c r="G2">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="3" spans="1:8" x14ac:dyDescent="0.2">
+      <c r="A3" s="1" t="s">
+        <v>4</v>
+      </c>
+      <c r="B3" t="s">
+        <v>5</v>
+      </c>
+      <c r="C3" t="s">
+        <v>15</v>
+      </c>
+      <c r="D3" t="s">
+        <v>10</v>
+      </c>
+      <c r="E3">
+        <v>976633782</v>
+      </c>
+      <c r="F3" t="s">
+        <v>8</v>
+      </c>
+      <c r="G3">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="4" spans="1:8" x14ac:dyDescent="0.2">
+      <c r="A4" t="s">
+        <v>16</v>
+      </c>
+      <c r="B4" t="s">
+        <v>18</v>
+      </c>
+      <c r="C4" t="s">
+        <v>17</v>
+      </c>
+      <c r="D4" t="s">
+        <v>10</v>
+      </c>
+      <c r="G4">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="5" spans="1:8" x14ac:dyDescent="0.2">
+      <c r="A5" t="s">
+        <v>19</v>
+      </c>
+      <c r="B5" t="s">
+        <v>20</v>
+      </c>
+      <c r="C5" t="s">
+        <v>21</v>
+      </c>
+      <c r="G5">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="6" spans="1:8" x14ac:dyDescent="0.2">
+      <c r="A6" t="s">
+        <v>22</v>
+      </c>
+      <c r="B6" t="s">
+        <v>23</v>
+      </c>
+      <c r="G6">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="7" spans="1:8" x14ac:dyDescent="0.2">
+      <c r="A7" t="s">
+        <v>24</v>
+      </c>
+      <c r="B7" t="s">
+        <v>25</v>
+      </c>
+      <c r="G7">
         <v>1</v>
       </c>
     </row>
   </sheetData>
   <hyperlinks>
     <hyperlink ref="A2" r:id="rId1" xr:uid="{B0D5F5F7-E548-9E4A-8E1A-429F8E3A939C}"/>
+    <hyperlink ref="A3" r:id="rId2" xr:uid="{E105403C-64B9-8D4C-ACE8-E89A3F2D4754}"/>
   </hyperlinks>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>